<commit_message>
Add more method for Table S6 / make Table S8 / reformat GalaxyWater-CNN data summary for easier reading
</commit_message>
<xml_diff>
--- a/manuscript_image/Table_S6.xlsx
+++ b/manuscript_image/Table_S6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\WatGNN_all\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\WatGNN_SI\manuscript_image\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C17A1C9B-3681-4107-8CA0-5115F249A0B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8056B9DA-2333-45E8-A95A-39AC0626EFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22860" yWindow="1680" windowWidth="23040" windowHeight="11295" xr2:uid="{4786BC20-B624-47F0-B5D0-ACF7443DB13D}"/>
+    <workbookView xWindow="120" yWindow="1470" windowWidth="18060" windowHeight="11295" xr2:uid="{4786BC20-B624-47F0-B5D0-ACF7443DB13D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
   <si>
     <t>Method</t>
   </si>
@@ -101,6 +101,94 @@
   </si>
   <si>
     <t>0.448 (0.150)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Single-protein Set</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GalaxyWater-CNN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3D-RISM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.288  (45.0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.448  (45.0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.481 (45.0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.355 (0.80)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.476 (0.70)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.516 (0.70)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.334 (45.0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.512 (45.0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.543 (42.5)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.327 (0.175)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.420 (0.125)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.442 (0.100)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.466 (8.00)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.396 (8.00)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.198 (8.00)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Protein-compound Set</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.118 (8.00)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.262 (8.00)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.344 (8.00)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -410,8 +498,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -419,13 +510,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -762,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97975BEB-6180-4361-B77A-D809BC9F1811}">
-  <dimension ref="F3:I10"/>
+  <dimension ref="F3:I21"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="6" max="6" width="11.125" customWidth="1"/>
@@ -771,20 +859,22 @@
   <sheetData>
     <row r="3" spans="6:9" ht="17.25" thickBot="1"/>
     <row r="4" spans="6:9" ht="18" customHeight="1" thickTop="1">
-      <c r="F4" s="10"/>
-      <c r="G4" s="11" t="s">
+      <c r="F4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="11"/>
-      <c r="I4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" spans="6:9" ht="22.5" customHeight="1" thickBot="1">
-      <c r="F5" s="13"/>
-      <c r="G5" s="14" t="s">
+      <c r="F5" s="15"/>
+      <c r="G5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="15"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" spans="6:9" ht="17.25" thickTop="1">
       <c r="F6" s="1" t="s">
@@ -814,40 +904,161 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="6:9" ht="30">
+    <row r="8" spans="6:9" ht="30" customHeight="1">
       <c r="F8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="6:9" ht="30" customHeight="1">
+      <c r="F9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="6:9" ht="30">
+      <c r="F10" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="6:9" ht="30.75" thickBot="1">
-      <c r="F9" s="7" t="s">
+    <row r="11" spans="6:9" ht="30.75" thickBot="1">
+      <c r="F11" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="6:9" ht="17.25" thickTop="1"/>
+    <row r="12" spans="6:9" ht="17.25" thickTop="1"/>
+    <row r="13" spans="6:9" ht="17.25" thickBot="1"/>
+    <row r="14" spans="6:9" ht="24.95" customHeight="1" thickTop="1">
+      <c r="F14" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="12"/>
+      <c r="I14" s="13"/>
+    </row>
+    <row r="15" spans="6:9" ht="20.100000000000001" customHeight="1" thickBot="1">
+      <c r="F15" s="15"/>
+      <c r="G15" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="10"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" spans="6:9" ht="17.25" thickTop="1">
+      <c r="F16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="6:9" ht="30">
+      <c r="F17" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="6:9" ht="30" customHeight="1">
+      <c r="F18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="6:9" ht="30">
+      <c r="F19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="6:9" ht="30.75" thickBot="1">
+      <c r="F20" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="6:9" ht="17.25" thickTop="1"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="F4:F5"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>